<commit_message>
Écran d'erreur explicite et import tolérant sur les noms de classe
- error.tsx : une page qui plante affiche un message clair, le détail
  technique et un bouton Réessayer, au lieu de « Application error »
- import : « 7e A », « 7ème A » et « 7e année A » désignent la même classe
  (nom exact prioritaire, forme courte seulement sans ambiguïté) ;
  le message d'erreur cite la classe introuvable et explique quoi faire
- fichier d'exemple aligné sur les classes créées par l'assistant

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012xbZc1XmQs8GsufaHyxYdk
</commit_message>
<xml_diff>
--- a/exemples/import-eleves-exemple.xlsx
+++ b/exemples/import-eleves-exemple.xlsx
@@ -62,7 +62,7 @@
     <t>Koutiala</t>
   </si>
   <si>
-    <t>7e A</t>
+    <t>7e année A</t>
   </si>
   <si>
     <t>Salimata</t>
@@ -224,7 +224,7 @@
     <t>22/12/2013</t>
   </si>
   <si>
-    <t>8e A</t>
+    <t>8e année A</t>
   </si>
   <si>
     <t>Rokia</t>
@@ -326,7 +326,7 @@
     <t>22/08/2012</t>
   </si>
   <si>
-    <t>9e A</t>
+    <t>9e année A</t>
   </si>
   <si>
     <t>70 00 01 24</t>
@@ -401,7 +401,7 @@
     <t>Fichier d'exemple pour tester l'import des élèves dans LAKOL (30 élèves fictifs).</t>
   </si>
   <si>
-    <t>AVANT L'IMPORT : créer dans LAKOL les classes « 7e A », « 8e A » et « 9e A » pour l'année scolaire active,</t>
+    <t>AVANT L'IMPORT : les classes « 7e année A », « 8e année A » et « 9e année A » doivent exister (l'assistant de démarrage les crée : cycle « Fondamental 2e cycle »),</t>
   </si>
   <si>
     <t>ou remplacer la colonne « classe » par les noms exacts de vos classes.</t>
@@ -819,7 +819,7 @@
     <col min="1" max="2" width="14" style="1" customWidth="1"/>
     <col min="3" max="3" width="6" style="1" customWidth="1"/>
     <col min="4" max="5" width="15" style="1" customWidth="1"/>
-    <col min="6" max="6" width="8" style="1" customWidth="1"/>
+    <col min="6" max="6" width="12" style="1" customWidth="1"/>
     <col min="7" max="8" width="14" style="1" customWidth="1"/>
     <col min="9" max="9" width="17" style="1" customWidth="1"/>
     <col min="10" max="10" width="28" style="1" customWidth="1"/>

</xml_diff>